<commit_message>
Add validation script for Excel and PUML files
- Implemented `check_excel_col` function to validate columns in Excel files against expected types, nullability, keys, and descriptions.
- Implemented `check_puml` function to validate patterns in PUML files.
- Added checks for various domains including user_roles, locations, sku_uom_conversions, sku_barcodes, sku_suppliers, inventory, stock_ledger, and audit.
- Collect validation results in a report and print summary of checks.
</commit_message>
<xml_diff>
--- a/tuan-02/Domain A/Data Dictionary domain A.xlsx
+++ b/tuan-02/Domain A/Data Dictionary domain A.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Domain A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Domain A" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1635,48 +1635,52 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>user_roles</t>
         </is>
       </c>
-      <c r="B35" s="6" t="inlineStr">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>BIGINT</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>PK</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Primary key</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>user_roles</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
         <is>
           <t>user_id</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>BIGINT</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="6" t="inlineStr">
-        <is>
-          <t>PK, FK → users.id</t>
-        </is>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>Người dùng được gán vai trò</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>role_id</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
@@ -1692,17 +1696,17 @@
       <c r="E36" s="6" t="n"/>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>PK, FK → roles.id</t>
+          <t>FK → users.id</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>Vai trò được gán</t>
+          <t>Người dùng được gán vai trò</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1714,7 @@
       <c r="A37" s="6" t="n"/>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>warehouse_id</t>
+          <t>role_id</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
@@ -1720,23 +1724,23 @@
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="E37" s="6" t="n"/>
       <c r="F37" s="6" t="inlineStr">
         <is>
-          <t>PK, FK → warehouses.id (domain B)</t>
+          <t>PK, FK → roles.id</t>
         </is>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Kho phạm vi; NULL = toàn hệ thống (ADMIN)</t>
+          <t>Vai trò được gán</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
     </row>
@@ -1744,31 +1748,33 @@
       <c r="A38" s="6" t="n"/>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>warehouse_id</t>
         </is>
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>BOOLEAN</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E38" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F38" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="n"/>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>PK, FK → warehouses.id (domain B)</t>
+        </is>
+      </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>Gán vai trò còn hiệu lực</t>
+          <t>Kho phạm vi; NULL = toàn hệ thống (ADMIN)</t>
         </is>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>true</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1776,12 +1782,12 @@
       <c r="A39" s="6" t="n"/>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>is_active</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
+          <t>BOOLEAN</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -1789,20 +1795,18 @@
           <t>N</t>
         </is>
       </c>
-      <c r="E39" s="6" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
+      <c r="E39" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F39" s="6" t="n"/>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm gán</t>
+          <t>Gán vai trò còn hiệu lực</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>2026-09-23 08:00:00</t>
+          <t>true</t>
         </is>
       </c>
     </row>
@@ -1810,12 +1814,12 @@
       <c r="A40" s="6" t="n"/>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>created_by</t>
+          <t>created_at</t>
         </is>
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>BIGINT</t>
+          <t>TIMESTAMP</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
@@ -1823,20 +1827,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="E40" s="6" t="n"/>
-      <c r="F40" s="6" t="inlineStr">
-        <is>
-          <t>FK → users.id</t>
-        </is>
-      </c>
+      <c r="E40" s="6" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="F40" s="6" t="n"/>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Người thực hiện gán (ADMIN)</t>
+          <t>Thời điểm gán</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2026-09-23 08:00:00</t>
         </is>
       </c>
     </row>
@@ -1844,12 +1848,12 @@
       <c r="A41" s="6" t="n"/>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>created_by</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>TIMESTAMP</t>
+          <t>BIGINT</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -1857,20 +1861,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="E41" s="6" t="inlineStr">
-        <is>
-          <t>now()</t>
-        </is>
-      </c>
-      <c r="F41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>FK → users.id</t>
+        </is>
+      </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Thời điểm cập nhật</t>
+          <t>Người thực hiện gán (ADMIN)</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>2026-09-23 08:00:00</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1878,31 +1882,65 @@
       <c r="A42" s="6" t="n"/>
       <c r="B42" s="6" t="inlineStr">
         <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>TIMESTAMP</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E42" s="6" t="inlineStr">
+        <is>
+          <t>now()</t>
+        </is>
+      </c>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>Thời điểm cập nhật</t>
+        </is>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-23 08:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n"/>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
           <t>updated_by</t>
         </is>
       </c>
-      <c r="C42" s="6" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>BIGINT</t>
         </is>
       </c>
-      <c r="D42" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="n"/>
-      <c r="F42" s="6" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="inlineStr">
         <is>
           <t>FK → users.id</t>
         </is>
       </c>
-      <c r="G42" s="6" t="inlineStr">
+      <c r="G43" s="6" t="inlineStr">
         <is>
           <t>Người cập nhật</t>
         </is>
       </c>
-      <c r="H42" s="6" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>

</xml_diff>